<commit_message>
add qc checklists, document expiry tracking, anniversary alerts wiring
</commit_message>
<xml_diff>
--- a/JAMM_PX_Master_Roadmap_v1.xlsx
+++ b/JAMM_PX_Master_Roadmap_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andre\Downloads\JAMM-Media\JAMM OS Build\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{067F2FCE-F237-4F59-A095-D8400A0F8625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAD5AA35-6952-4067-8EB4-F4B4486D01A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AI Instructions" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1596" uniqueCount="866">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1597" uniqueCount="868">
   <si>
     <t>JAMM PX — Session Build Status</t>
   </si>
@@ -2693,6 +2693,12 @@
   </si>
   <si>
     <t>Consistent vocabulary throughout UI and codebase.</t>
+  </si>
+  <si>
+    <t>13A - Tax Practice+A5:G42</t>
+  </si>
+  <si>
+    <t>index analytics agent</t>
   </si>
 </sst>
 </file>
@@ -3109,15 +3115,24 @@
     <xf numFmtId="0" fontId="4" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3125,20 +3140,11 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3450,139 +3456,139 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="68" t="s">
         <v>112</v>
       </c>
       <c r="B1" s="60"/>
     </row>
     <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="67" t="s">
         <v>113</v>
       </c>
       <c r="B2" s="60"/>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="65" t="s">
         <v>114</v>
       </c>
       <c r="B3" s="60"/>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="66" t="s">
         <v>115</v>
       </c>
       <c r="B4" s="60"/>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A5" s="61" t="s">
+      <c r="A5" s="65" t="s">
         <v>116</v>
       </c>
       <c r="B5" s="60"/>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A6" s="63" t="s">
+      <c r="A6" s="66" t="s">
         <v>117</v>
       </c>
       <c r="B6" s="60"/>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A7" s="61" t="s">
+      <c r="A7" s="65" t="s">
         <v>118</v>
       </c>
       <c r="B7" s="60"/>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A8" s="63" t="s">
+      <c r="A8" s="66" t="s">
         <v>119</v>
       </c>
       <c r="B8" s="60"/>
     </row>
     <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A9" s="61" t="s">
+      <c r="A9" s="65" t="s">
         <v>120</v>
       </c>
       <c r="B9" s="60"/>
     </row>
     <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A10" s="63" t="s">
+      <c r="A10" s="66" t="s">
         <v>121</v>
       </c>
       <c r="B10" s="60"/>
     </row>
     <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A11" s="61" t="s">
+      <c r="A11" s="65" t="s">
         <v>122</v>
       </c>
       <c r="B11" s="60"/>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A12" s="64" t="s">
+      <c r="A12" s="67" t="s">
         <v>123</v>
       </c>
       <c r="B12" s="60"/>
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A13" s="61" t="s">
+      <c r="A13" s="65" t="s">
         <v>124</v>
       </c>
       <c r="B13" s="60"/>
     </row>
     <row r="14" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A14" s="64" t="s">
+      <c r="A14" s="67" t="s">
         <v>125</v>
       </c>
       <c r="B14" s="60"/>
     </row>
     <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A15" s="61" t="s">
+      <c r="A15" s="65" t="s">
         <v>126</v>
       </c>
       <c r="B15" s="60"/>
     </row>
     <row r="16" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A16" s="64" t="s">
+      <c r="A16" s="67" t="s">
         <v>127</v>
       </c>
       <c r="B16" s="60"/>
     </row>
     <row r="17" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A17" s="61" t="s">
+      <c r="A17" s="65" t="s">
         <v>128</v>
       </c>
       <c r="B17" s="60"/>
     </row>
     <row r="18" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A18" s="64" t="s">
+      <c r="A18" s="67" t="s">
         <v>129</v>
       </c>
       <c r="B18" s="60"/>
     </row>
     <row r="19" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A19" s="61" t="s">
+      <c r="A19" s="65" t="s">
         <v>130</v>
       </c>
       <c r="B19" s="60"/>
     </row>
     <row r="20" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A20" s="64" t="s">
+      <c r="A20" s="67" t="s">
         <v>131</v>
       </c>
       <c r="B20" s="60"/>
     </row>
     <row r="21" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A21" s="61" t="s">
+      <c r="A21" s="65" t="s">
         <v>132</v>
       </c>
       <c r="B21" s="60"/>
     </row>
     <row r="22" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A22" s="64" t="s">
+      <c r="A22" s="67" t="s">
         <v>133</v>
       </c>
       <c r="B22" s="60"/>
     </row>
     <row r="23" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A23" s="61" t="s">
+      <c r="A23" s="65" t="s">
         <v>134</v>
       </c>
       <c r="B23" s="60"/>
@@ -3619,6 +3625,18 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A11:B11"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A8:B8"/>
@@ -3630,18 +3648,6 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A7:B7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3661,7 +3667,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="63" t="s">
         <v>141</v>
       </c>
       <c r="B1" s="60"/>
@@ -3695,7 +3701,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A3" s="65" t="s">
+      <c r="A3" s="62" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="60"/>
@@ -4695,7 +4701,7 @@
       </c>
     </row>
     <row r="47" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A47" s="69" t="s">
+      <c r="A47" s="64" t="s">
         <v>273</v>
       </c>
       <c r="B47" s="60"/>
@@ -4798,7 +4804,7 @@
       </c>
     </row>
     <row r="52" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A52" s="68" t="s">
+      <c r="A52" s="61" t="s">
         <v>102</v>
       </c>
       <c r="B52" s="60"/>
@@ -4809,7 +4815,7 @@
       <c r="G52" s="60"/>
     </row>
     <row r="53" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A53" s="65" t="s">
+      <c r="A53" s="62" t="s">
         <v>13</v>
       </c>
       <c r="B53" s="60"/>
@@ -4866,7 +4872,7 @@
       </c>
     </row>
     <row r="56" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A56" s="65" t="s">
+      <c r="A56" s="62" t="s">
         <v>13</v>
       </c>
       <c r="B56" s="60"/>
@@ -4969,7 +4975,7 @@
       </c>
     </row>
     <row r="61" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A61" s="65" t="s">
+      <c r="A61" s="62" t="s">
         <v>13</v>
       </c>
       <c r="B61" s="60"/>
@@ -5003,7 +5009,7 @@
       </c>
     </row>
     <row r="63" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A63" s="65" t="s">
+      <c r="A63" s="62" t="s">
         <v>13</v>
       </c>
       <c r="B63" s="60"/>
@@ -5037,7 +5043,7 @@
       </c>
     </row>
     <row r="65" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A65" s="65" t="s">
+      <c r="A65" s="62" t="s">
         <v>13</v>
       </c>
       <c r="B65" s="60"/>
@@ -5117,7 +5123,7 @@
       </c>
     </row>
     <row r="69" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A69" s="67" t="s">
+      <c r="A69" s="59" t="s">
         <v>325</v>
       </c>
       <c r="B69" s="60"/>
@@ -5151,7 +5157,7 @@
       </c>
     </row>
     <row r="71" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A71" s="68" t="s">
+      <c r="A71" s="61" t="s">
         <v>102</v>
       </c>
       <c r="B71" s="60"/>
@@ -5255,17 +5261,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A56:G56"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A53:G53"/>
+    <mergeCell ref="A47:G47"/>
     <mergeCell ref="A69:G69"/>
     <mergeCell ref="A52:G52"/>
     <mergeCell ref="A65:G65"/>
     <mergeCell ref="A71:G71"/>
     <mergeCell ref="A63:G63"/>
     <mergeCell ref="A61:G61"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A56:G56"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A53:G53"/>
-    <mergeCell ref="A47:G47"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5287,7 +5293,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="68" t="s">
         <v>339</v>
       </c>
       <c r="B1" s="60"/>
@@ -5325,7 +5331,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A3" s="69" t="s">
+      <c r="A3" s="64" t="s">
         <v>345</v>
       </c>
       <c r="B3" s="60"/>
@@ -5433,7 +5439,7 @@
       <c r="H7" s="6"/>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A8" s="69" t="s">
+      <c r="A8" s="64" t="s">
         <v>361</v>
       </c>
       <c r="B8" s="60"/>
@@ -5695,7 +5701,7 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A19" s="69" t="s">
+      <c r="A19" s="64" t="s">
         <v>404</v>
       </c>
       <c r="B19" s="60"/>
@@ -5857,7 +5863,7 @@
       </c>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A26" s="69" t="s">
+      <c r="A26" s="64" t="s">
         <v>433</v>
       </c>
       <c r="B26" s="60"/>
@@ -5943,7 +5949,7 @@
       <c r="H29" s="6"/>
     </row>
     <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A30" s="69" t="s">
+      <c r="A30" s="64" t="s">
         <v>445</v>
       </c>
       <c r="B30" s="60"/>
@@ -6027,7 +6033,7 @@
       <c r="H33" s="6"/>
     </row>
     <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A34" s="69" t="s">
+      <c r="A34" s="64" t="s">
         <v>458</v>
       </c>
       <c r="B34" s="60"/>
@@ -6285,7 +6291,7 @@
       </c>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A45" s="69" t="s">
+      <c r="A45" s="64" t="s">
         <v>498</v>
       </c>
       <c r="B45" s="60"/>
@@ -6471,7 +6477,7 @@
       </c>
     </row>
     <row r="53" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A53" s="69" t="s">
+      <c r="A53" s="64" t="s">
         <v>530</v>
       </c>
       <c r="B53" s="60"/>
@@ -6507,7 +6513,7 @@
       <c r="H54" s="5"/>
     </row>
     <row r="55" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A55" s="69" t="s">
+      <c r="A55" s="64" t="s">
         <v>535</v>
       </c>
       <c r="B55" s="60"/>
@@ -6600,7 +6606,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="68" t="s">
         <v>544</v>
       </c>
       <c r="B1" s="60"/>
@@ -6626,7 +6632,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A3" s="69" t="s">
+      <c r="A3" s="64" t="s">
         <v>549</v>
       </c>
       <c r="B3" s="60"/>
@@ -6788,7 +6794,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A13" s="69" t="s">
+      <c r="A13" s="64" t="s">
         <v>577</v>
       </c>
       <c r="B13" s="60"/>
@@ -6910,7 +6916,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -6923,7 +6929,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="68" t="s">
         <v>596</v>
       </c>
       <c r="B1" s="60"/>
@@ -6956,7 +6962,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A3" s="69" t="s">
+      <c r="A3" s="64" t="s">
         <v>599</v>
       </c>
       <c r="B3" s="60"/>
@@ -6994,7 +7000,7 @@
         <v>152</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>600</v>
+        <v>866</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>605</v>
@@ -7013,7 +7019,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A6" s="69" t="s">
+      <c r="A6" s="64" t="s">
         <v>609</v>
       </c>
       <c r="B6" s="60"/>
@@ -7093,7 +7099,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A10" s="69" t="s">
+      <c r="A10" s="64" t="s">
         <v>621</v>
       </c>
       <c r="B10" s="60"/>
@@ -7196,7 +7202,7 @@
       </c>
     </row>
     <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A15" s="69" t="s">
+      <c r="A15" s="64" t="s">
         <v>635</v>
       </c>
       <c r="B15" s="60"/>
@@ -7299,7 +7305,7 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A20" s="69" t="s">
+      <c r="A20" s="64" t="s">
         <v>647</v>
       </c>
       <c r="B20" s="60"/>
@@ -7402,7 +7408,7 @@
       </c>
     </row>
     <row r="25" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A25" s="69" t="s">
+      <c r="A25" s="64" t="s">
         <v>307</v>
       </c>
       <c r="B25" s="60"/>
@@ -7505,7 +7511,7 @@
       </c>
     </row>
     <row r="30" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A30" s="69" t="s">
+      <c r="A30" s="64" t="s">
         <v>674</v>
       </c>
       <c r="B30" s="60"/>
@@ -7562,7 +7568,7 @@
       </c>
     </row>
     <row r="33" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A33" s="69" t="s">
+      <c r="A33" s="64" t="s">
         <v>682</v>
       </c>
       <c r="B33" s="60"/>
@@ -7619,7 +7625,7 @@
       </c>
     </row>
     <row r="36" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A36" s="69" t="s">
+      <c r="A36" s="64" t="s">
         <v>691</v>
       </c>
       <c r="B36" s="60"/>
@@ -7699,7 +7705,7 @@
       </c>
     </row>
     <row r="40" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A40" s="69" t="s">
+      <c r="A40" s="64" t="s">
         <v>702</v>
       </c>
       <c r="B40" s="60"/>
@@ -7756,7 +7762,7 @@
       </c>
     </row>
     <row r="43" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A43" s="69" t="s">
+      <c r="A43" s="64" t="s">
         <v>711</v>
       </c>
       <c r="B43" s="60"/>
@@ -7789,13 +7795,13 @@
         <v>102</v>
       </c>
     </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="B46" t="s">
+        <v>867</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A43:G43"/>
-    <mergeCell ref="A33:G33"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A36:G36"/>
-    <mergeCell ref="A40:G40"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A6:G6"/>
     <mergeCell ref="A1:F1"/>
@@ -7803,6 +7809,11 @@
     <mergeCell ref="A30:G30"/>
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A40:G40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7824,7 +7835,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="69" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="60"/>
@@ -7836,7 +7847,7 @@
       <c r="H1" s="60"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="69" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="60"/>
@@ -8390,7 +8401,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="61" t="s">
         <v>102</v>
       </c>
       <c r="B1" s="60"/>
@@ -9002,7 +9013,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="68" t="s">
         <v>800</v>
       </c>
       <c r="B1" s="60"/>

</xml_diff>